<commit_message>
Add React web app, README, Excel templates and tidier sample data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017xi9tmff2aXUsJqNMSBAwk
</commit_message>
<xml_diff>
--- a/templates/SGUMC_Radiology_Schedule_Sample.xlsx
+++ b/templates/SGUMC_Radiology_Schedule_Sample.xlsx
@@ -2306,10 +2306,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="4">
-        <v>46510</v>
+        <v>46237</v>
       </c>
       <c r="D4" s="4">
-        <v>46521</v>
+        <v>46248</v>
       </c>
       <c r="E4" t="s">
         <v>80</v>
@@ -2340,10 +2340,10 @@
         <v>21</v>
       </c>
       <c r="C6" s="4">
-        <v>46449</v>
+        <v>46510</v>
       </c>
       <c r="D6" s="4">
-        <v>46460</v>
+        <v>46521</v>
       </c>
       <c r="E6" t="s">
         <v>80</v>
@@ -2357,10 +2357,10 @@
         <v>24</v>
       </c>
       <c r="C7" s="4">
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="D7" s="4">
-        <v>46255</v>
+        <v>46286</v>
       </c>
       <c r="E7" t="s">
         <v>80</v>
@@ -2374,10 +2374,10 @@
         <v>27</v>
       </c>
       <c r="C8" s="4">
-        <v>46390</v>
+        <v>46449</v>
       </c>
       <c r="D8" s="4">
-        <v>46401</v>
+        <v>46460</v>
       </c>
       <c r="E8" t="s">
         <v>79</v>
@@ -2408,10 +2408,10 @@
         <v>34</v>
       </c>
       <c r="C10" s="4">
-        <v>46329</v>
+        <v>46390</v>
       </c>
       <c r="D10" s="4">
-        <v>46340</v>
+        <v>46401</v>
       </c>
       <c r="E10" t="s">
         <v>80</v>
@@ -2442,10 +2442,10 @@
         <v>40</v>
       </c>
       <c r="C12" s="4">
-        <v>46268</v>
+        <v>46329</v>
       </c>
       <c r="D12" s="4">
-        <v>46279</v>
+        <v>46340</v>
       </c>
       <c r="E12" t="s">
         <v>80</v>
@@ -3036,10 +3036,10 @@
         <v>46245</v>
       </c>
       <c r="B43" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C43" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -3047,10 +3047,10 @@
         <v>46246</v>
       </c>
       <c r="B44" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C44" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -3058,10 +3058,10 @@
         <v>46247</v>
       </c>
       <c r="B45" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C45" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -3069,10 +3069,10 @@
         <v>46248</v>
       </c>
       <c r="B46" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C46" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -3080,10 +3080,10 @@
         <v>46249</v>
       </c>
       <c r="B47" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C47" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -3091,10 +3091,10 @@
         <v>46250</v>
       </c>
       <c r="B48" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C48" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -3102,10 +3102,10 @@
         <v>46251</v>
       </c>
       <c r="B49" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C49" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -3113,10 +3113,10 @@
         <v>46252</v>
       </c>
       <c r="B50" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C50" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -3124,10 +3124,10 @@
         <v>46253</v>
       </c>
       <c r="B51" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C51" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -3135,10 +3135,10 @@
         <v>46254</v>
       </c>
       <c r="B52" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C52" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -3146,10 +3146,10 @@
         <v>46255</v>
       </c>
       <c r="B53" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="C53" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -3157,10 +3157,10 @@
         <v>46256</v>
       </c>
       <c r="B54" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C54" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -3179,10 +3179,10 @@
         <v>46258</v>
       </c>
       <c r="B56" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C56" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -3190,10 +3190,10 @@
         <v>46259</v>
       </c>
       <c r="B57" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C57" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -3201,10 +3201,10 @@
         <v>46260</v>
       </c>
       <c r="B58" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C58" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -3212,10 +3212,10 @@
         <v>46261</v>
       </c>
       <c r="B59" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C59" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -3223,10 +3223,10 @@
         <v>46262</v>
       </c>
       <c r="B60" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C60" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -3234,10 +3234,10 @@
         <v>46263</v>
       </c>
       <c r="B61" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C61" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -3245,10 +3245,10 @@
         <v>46264</v>
       </c>
       <c r="B62" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C62" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -3256,10 +3256,10 @@
         <v>46265</v>
       </c>
       <c r="B63" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C63" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -3278,10 +3278,10 @@
         <v>46267</v>
       </c>
       <c r="B65" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="C65" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -3289,10 +3289,10 @@
         <v>46268</v>
       </c>
       <c r="B66" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="C66" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -3300,10 +3300,10 @@
         <v>46269</v>
       </c>
       <c r="B67" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C67" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -3322,10 +3322,10 @@
         <v>46271</v>
       </c>
       <c r="B69" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C69" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -3333,10 +3333,10 @@
         <v>46272</v>
       </c>
       <c r="B70" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C70" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -3344,10 +3344,10 @@
         <v>46273</v>
       </c>
       <c r="B71" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C71" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -3355,10 +3355,10 @@
         <v>46274</v>
       </c>
       <c r="B72" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="C72" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -3399,10 +3399,10 @@
         <v>46278</v>
       </c>
       <c r="B76" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C76" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -3410,10 +3410,10 @@
         <v>46279</v>
       </c>
       <c r="B77" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C77" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -3443,10 +3443,10 @@
         <v>46282</v>
       </c>
       <c r="B80" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C80" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -3454,10 +3454,10 @@
         <v>46283</v>
       </c>
       <c r="B81" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C81" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -3465,10 +3465,10 @@
         <v>46284</v>
       </c>
       <c r="B82" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C82" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -3476,10 +3476,10 @@
         <v>46285</v>
       </c>
       <c r="B83" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="C83" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -3487,10 +3487,10 @@
         <v>46286</v>
       </c>
       <c r="B84" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C84" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -3498,10 +3498,10 @@
         <v>46287</v>
       </c>
       <c r="B85" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C85" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -3542,10 +3542,10 @@
         <v>46291</v>
       </c>
       <c r="B89" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C89" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -3553,10 +3553,10 @@
         <v>46292</v>
       </c>
       <c r="B90" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C90" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -3586,10 +3586,10 @@
         <v>46295</v>
       </c>
       <c r="B93" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C93" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -3608,10 +3608,10 @@
         <v>46297</v>
       </c>
       <c r="B95" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C95" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
@@ -3619,10 +3619,10 @@
         <v>46298</v>
       </c>
       <c r="B96" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C96" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
@@ -3630,10 +3630,10 @@
         <v>46299</v>
       </c>
       <c r="B97" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="C97" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
@@ -3641,10 +3641,10 @@
         <v>46300</v>
       </c>
       <c r="B98" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C98" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
@@ -3652,10 +3652,10 @@
         <v>46301</v>
       </c>
       <c r="B99" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C99" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -3729,10 +3729,10 @@
         <v>46308</v>
       </c>
       <c r="B106" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C106" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -3751,10 +3751,10 @@
         <v>46310</v>
       </c>
       <c r="B108" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C108" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -3762,10 +3762,10 @@
         <v>46311</v>
       </c>
       <c r="B109" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C109" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
@@ -3773,10 +3773,10 @@
         <v>46312</v>
       </c>
       <c r="B110" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C110" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
@@ -3784,10 +3784,10 @@
         <v>46313</v>
       </c>
       <c r="B111" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C111" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
@@ -3872,10 +3872,10 @@
         <v>46321</v>
       </c>
       <c r="B119" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C119" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
@@ -3894,10 +3894,10 @@
         <v>46323</v>
       </c>
       <c r="B121" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C121" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
@@ -3905,10 +3905,10 @@
         <v>46324</v>
       </c>
       <c r="B122" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C122" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
@@ -3916,10 +3916,10 @@
         <v>46325</v>
       </c>
       <c r="B123" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C123" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
@@ -3927,10 +3927,10 @@
         <v>46326</v>
       </c>
       <c r="B124" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C124" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
@@ -4015,10 +4015,10 @@
         <v>46334</v>
       </c>
       <c r="B132" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C132" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
@@ -4026,10 +4026,10 @@
         <v>46335</v>
       </c>
       <c r="B133" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C133" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -4037,10 +4037,10 @@
         <v>46336</v>
       </c>
       <c r="B134" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C134" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -4059,10 +4059,10 @@
         <v>46338</v>
       </c>
       <c r="B136" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C136" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
@@ -4070,10 +4070,10 @@
         <v>46339</v>
       </c>
       <c r="B137" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C137" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
@@ -4081,10 +4081,10 @@
         <v>46340</v>
       </c>
       <c r="B138" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C138" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
@@ -4092,10 +4092,10 @@
         <v>46341</v>
       </c>
       <c r="B139" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C139" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
@@ -4158,10 +4158,10 @@
         <v>46347</v>
       </c>
       <c r="B145" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C145" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
@@ -4169,10 +4169,10 @@
         <v>46348</v>
       </c>
       <c r="B146" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C146" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
@@ -4180,10 +4180,10 @@
         <v>46349</v>
       </c>
       <c r="B147" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C147" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
@@ -4202,10 +4202,10 @@
         <v>46351</v>
       </c>
       <c r="B149" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C149" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
@@ -4213,10 +4213,10 @@
         <v>46352</v>
       </c>
       <c r="B150" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C150" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
@@ -4224,10 +4224,10 @@
         <v>46353</v>
       </c>
       <c r="B151" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C151" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
@@ -4235,10 +4235,10 @@
         <v>46354</v>
       </c>
       <c r="B152" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
@@ -4312,10 +4312,10 @@
         <v>46361</v>
       </c>
       <c r="B159" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C159" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
@@ -4323,10 +4323,10 @@
         <v>46362</v>
       </c>
       <c r="B160" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C160" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
@@ -4334,10 +4334,10 @@
         <v>46363</v>
       </c>
       <c r="B161" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C161" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
@@ -4356,10 +4356,10 @@
         <v>46365</v>
       </c>
       <c r="B163" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C163" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
@@ -4367,10 +4367,10 @@
         <v>46366</v>
       </c>
       <c r="B164" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C164" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
@@ -4378,10 +4378,10 @@
         <v>46367</v>
       </c>
       <c r="B165" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C165" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
@@ -4389,10 +4389,10 @@
         <v>46368</v>
       </c>
       <c r="B166" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
@@ -4433,10 +4433,10 @@
         <v>46372</v>
       </c>
       <c r="B170" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C170" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
@@ -4444,10 +4444,10 @@
         <v>46373</v>
       </c>
       <c r="B171" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C171" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
@@ -4455,10 +4455,10 @@
         <v>46374</v>
       </c>
       <c r="B172" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C172" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
@@ -4477,10 +4477,10 @@
         <v>46376</v>
       </c>
       <c r="B174" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C174" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
@@ -4488,10 +4488,10 @@
         <v>46377</v>
       </c>
       <c r="B175" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C175" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
@@ -4521,10 +4521,10 @@
         <v>46380</v>
       </c>
       <c r="B178" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C178" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
@@ -4532,10 +4532,10 @@
         <v>46381</v>
       </c>
       <c r="B179" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C179" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
@@ -4576,10 +4576,10 @@
         <v>46385</v>
       </c>
       <c r="B183" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C183" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
@@ -4587,10 +4587,10 @@
         <v>46386</v>
       </c>
       <c r="B184" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C184" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
@@ -4598,10 +4598,10 @@
         <v>46387</v>
       </c>
       <c r="B185" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C185" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
@@ -4631,10 +4631,10 @@
         <v>46390</v>
       </c>
       <c r="B188" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C188" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
@@ -4642,10 +4642,10 @@
         <v>46391</v>
       </c>
       <c r="B189" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C189" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
@@ -4675,10 +4675,10 @@
         <v>46394</v>
       </c>
       <c r="B192" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C192" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -4697,10 +4697,10 @@
         <v>46396</v>
       </c>
       <c r="B194" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C194" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
@@ -4708,10 +4708,10 @@
         <v>46397</v>
       </c>
       <c r="B195" t="s">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="C195" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
@@ -4719,10 +4719,10 @@
         <v>46398</v>
       </c>
       <c r="B196" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C196" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
@@ -4730,10 +4730,10 @@
         <v>46399</v>
       </c>
       <c r="B197" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C197" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
@@ -4741,10 +4741,10 @@
         <v>46400</v>
       </c>
       <c r="B198" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="C198" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
@@ -4752,10 +4752,10 @@
         <v>46401</v>
       </c>
       <c r="B199" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C199" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
@@ -4763,10 +4763,10 @@
         <v>46402</v>
       </c>
       <c r="B200" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C200" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
@@ -4774,10 +4774,10 @@
         <v>46403</v>
       </c>
       <c r="B201" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C201" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
@@ -4785,10 +4785,10 @@
         <v>46404</v>
       </c>
       <c r="B202" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C202" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
@@ -4818,10 +4818,10 @@
         <v>46407</v>
       </c>
       <c r="B205" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C205" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
@@ -4840,10 +4840,10 @@
         <v>46409</v>
       </c>
       <c r="B207" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C207" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
@@ -4851,10 +4851,10 @@
         <v>46410</v>
       </c>
       <c r="B208" t="s">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="C208" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
@@ -4862,10 +4862,10 @@
         <v>46411</v>
       </c>
       <c r="B209" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C209" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
@@ -4873,10 +4873,10 @@
         <v>46412</v>
       </c>
       <c r="B210" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C210" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
@@ -4884,10 +4884,10 @@
         <v>46413</v>
       </c>
       <c r="B211" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="C211" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
@@ -4895,10 +4895,10 @@
         <v>46414</v>
       </c>
       <c r="B212" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C212" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
@@ -4906,10 +4906,10 @@
         <v>46415</v>
       </c>
       <c r="B213" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C213" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
@@ -4917,10 +4917,10 @@
         <v>46416</v>
       </c>
       <c r="B214" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C214" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
@@ -4928,10 +4928,10 @@
         <v>46417</v>
       </c>
       <c r="B215" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C215" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
@@ -4961,10 +4961,10 @@
         <v>46420</v>
       </c>
       <c r="B218" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C218" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
@@ -4983,10 +4983,10 @@
         <v>46422</v>
       </c>
       <c r="B220" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C220" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
@@ -4994,10 +4994,10 @@
         <v>46423</v>
       </c>
       <c r="B221" t="s">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="C221" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
@@ -5005,10 +5005,10 @@
         <v>46424</v>
       </c>
       <c r="B222" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C222" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
@@ -5016,10 +5016,10 @@
         <v>46425</v>
       </c>
       <c r="B223" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C223" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
@@ -5049,10 +5049,10 @@
         <v>46428</v>
       </c>
       <c r="B226" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C226" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
@@ -5060,10 +5060,10 @@
         <v>46429</v>
       </c>
       <c r="B227" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C227" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
@@ -5093,10 +5093,10 @@
         <v>46432</v>
       </c>
       <c r="B230" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C230" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
@@ -5115,10 +5115,10 @@
         <v>46434</v>
       </c>
       <c r="B232" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C232" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
@@ -5126,10 +5126,10 @@
         <v>46435</v>
       </c>
       <c r="B233" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C233" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
@@ -5137,10 +5137,10 @@
         <v>46436</v>
       </c>
       <c r="B234" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C234" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
@@ -5170,10 +5170,10 @@
         <v>46439</v>
       </c>
       <c r="B237" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C237" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
@@ -5192,10 +5192,10 @@
         <v>46441</v>
       </c>
       <c r="B239" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C239" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
@@ -5225,10 +5225,10 @@
         <v>46444</v>
       </c>
       <c r="B242" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C242" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
@@ -5247,10 +5247,10 @@
         <v>46446</v>
       </c>
       <c r="B244" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C244" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
@@ -5269,10 +5269,10 @@
         <v>46448</v>
       </c>
       <c r="B246" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C246" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
@@ -5280,10 +5280,10 @@
         <v>46449</v>
       </c>
       <c r="B247" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="C247" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
@@ -5291,10 +5291,10 @@
         <v>46450</v>
       </c>
       <c r="B248" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C248" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
@@ -5302,10 +5302,10 @@
         <v>46451</v>
       </c>
       <c r="B249" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C249" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
@@ -5324,10 +5324,10 @@
         <v>46453</v>
       </c>
       <c r="B251" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C251" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
@@ -5357,10 +5357,10 @@
         <v>46456</v>
       </c>
       <c r="B254" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C254" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
@@ -5379,10 +5379,10 @@
         <v>46458</v>
       </c>
       <c r="B256" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C256" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
@@ -5390,10 +5390,10 @@
         <v>46459</v>
       </c>
       <c r="B257" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C257" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
@@ -5401,10 +5401,10 @@
         <v>46460</v>
       </c>
       <c r="B258" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C258" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
@@ -5412,10 +5412,10 @@
         <v>46461</v>
       </c>
       <c r="B259" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="C259" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
@@ -5423,10 +5423,10 @@
         <v>46462</v>
       </c>
       <c r="B260" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C260" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
@@ -5434,10 +5434,10 @@
         <v>46463</v>
       </c>
       <c r="B261" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C261" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
@@ -5456,10 +5456,10 @@
         <v>46465</v>
       </c>
       <c r="B263" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C263" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
@@ -5489,10 +5489,10 @@
         <v>46468</v>
       </c>
       <c r="B266" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C266" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
@@ -5511,10 +5511,10 @@
         <v>46470</v>
       </c>
       <c r="B268" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C268" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
@@ -5522,10 +5522,10 @@
         <v>46471</v>
       </c>
       <c r="B269" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C269" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
@@ -5533,10 +5533,10 @@
         <v>46472</v>
       </c>
       <c r="B270" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C270" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
@@ -5544,10 +5544,10 @@
         <v>46473</v>
       </c>
       <c r="B271" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="C271" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
@@ -5555,10 +5555,10 @@
         <v>46474</v>
       </c>
       <c r="B272" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C272" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
@@ -5566,10 +5566,10 @@
         <v>46475</v>
       </c>
       <c r="B273" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C273" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
@@ -5588,10 +5588,10 @@
         <v>46477</v>
       </c>
       <c r="B275" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C275" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
@@ -5632,10 +5632,10 @@
         <v>46481</v>
       </c>
       <c r="B279" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C279" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
@@ -5643,10 +5643,10 @@
         <v>46482</v>
       </c>
       <c r="B280" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C280" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
@@ -5654,10 +5654,10 @@
         <v>46483</v>
       </c>
       <c r="B281" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C281" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
@@ -5665,10 +5665,10 @@
         <v>46484</v>
       </c>
       <c r="B282" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C282" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
@@ -5676,10 +5676,10 @@
         <v>46485</v>
       </c>
       <c r="B283" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="C283" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
@@ -5687,10 +5687,10 @@
         <v>46486</v>
       </c>
       <c r="B284" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C284" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
@@ -5698,10 +5698,10 @@
         <v>46487</v>
       </c>
       <c r="B285" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C285" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
@@ -5720,10 +5720,10 @@
         <v>46489</v>
       </c>
       <c r="B287" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C287" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.25">
@@ -5731,10 +5731,10 @@
         <v>46490</v>
       </c>
       <c r="B288" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C288" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
@@ -5742,10 +5742,10 @@
         <v>46491</v>
       </c>
       <c r="B289" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="C289" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
@@ -5753,10 +5753,10 @@
         <v>46492</v>
       </c>
       <c r="B290" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C290" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.25">
@@ -5764,10 +5764,10 @@
         <v>46493</v>
       </c>
       <c r="B291" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C291" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
@@ -5775,10 +5775,10 @@
         <v>46494</v>
       </c>
       <c r="B292" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C292" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
@@ -5786,10 +5786,10 @@
         <v>46495</v>
       </c>
       <c r="B293" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C293" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="294" spans="1:3" x14ac:dyDescent="0.25">
@@ -5797,10 +5797,10 @@
         <v>46496</v>
       </c>
       <c r="B294" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="C294" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
@@ -5808,10 +5808,10 @@
         <v>46497</v>
       </c>
       <c r="B295" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C295" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.25">
@@ -5819,10 +5819,10 @@
         <v>46498</v>
       </c>
       <c r="B296" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C296" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.25">
@@ -5852,10 +5852,10 @@
         <v>46501</v>
       </c>
       <c r="B299" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C299" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.25">
@@ -5863,10 +5863,10 @@
         <v>46502</v>
       </c>
       <c r="B300" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C300" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.25">
@@ -5874,10 +5874,10 @@
         <v>46503</v>
       </c>
       <c r="B301" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="C301" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.25">
@@ -5885,10 +5885,10 @@
         <v>46504</v>
       </c>
       <c r="B302" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C302" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
     </row>
     <row r="303" spans="1:3" x14ac:dyDescent="0.25">
@@ -5896,10 +5896,10 @@
         <v>46505</v>
       </c>
       <c r="B303" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C303" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.25">
@@ -5907,10 +5907,10 @@
         <v>46506</v>
       </c>
       <c r="B304" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C304" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.25">
@@ -5918,10 +5918,10 @@
         <v>46507</v>
       </c>
       <c r="B305" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C305" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
@@ -5940,10 +5940,10 @@
         <v>46509</v>
       </c>
       <c r="B307" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="C307" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.25">
@@ -5951,10 +5951,10 @@
         <v>46510</v>
       </c>
       <c r="B308" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C308" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.25">
@@ -5984,10 +5984,10 @@
         <v>46513</v>
       </c>
       <c r="B311" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C311" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.25">
@@ -5995,10 +5995,10 @@
         <v>46514</v>
       </c>
       <c r="B312" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C312" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.25">
@@ -6006,10 +6006,10 @@
         <v>46515</v>
       </c>
       <c r="B313" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="C313" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.25">
@@ -6017,10 +6017,10 @@
         <v>46516</v>
       </c>
       <c r="B314" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C314" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
@@ -6028,10 +6028,10 @@
         <v>46517</v>
       </c>
       <c r="B315" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C315" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.25">
@@ -6039,10 +6039,10 @@
         <v>46518</v>
       </c>
       <c r="B316" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C316" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.25">
@@ -6050,10 +6050,10 @@
         <v>46519</v>
       </c>
       <c r="B317" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C317" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.25">
@@ -6061,10 +6061,10 @@
         <v>46520</v>
       </c>
       <c r="B318" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C318" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.25">
@@ -6072,10 +6072,10 @@
         <v>46521</v>
       </c>
       <c r="B319" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C319" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.25">
@@ -6083,10 +6083,10 @@
         <v>46522</v>
       </c>
       <c r="B320" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C320" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.25">
@@ -6116,10 +6116,10 @@
         <v>46525</v>
       </c>
       <c r="B323" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C323" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.25">
@@ -6127,10 +6127,10 @@
         <v>46526</v>
       </c>
       <c r="B324" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C324" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.25">
@@ -6138,10 +6138,10 @@
         <v>46527</v>
       </c>
       <c r="B325" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="C325" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.25">
@@ -6149,10 +6149,10 @@
         <v>46528</v>
       </c>
       <c r="B326" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C326" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
     </row>
     <row r="327" spans="1:3" x14ac:dyDescent="0.25">
@@ -6160,10 +6160,10 @@
         <v>46529</v>
       </c>
       <c r="B327" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C327" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="328" spans="1:3" x14ac:dyDescent="0.25">
@@ -6171,10 +6171,10 @@
         <v>46530</v>
       </c>
       <c r="B328" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C328" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="329" spans="1:3" x14ac:dyDescent="0.25">
@@ -6182,10 +6182,10 @@
         <v>46531</v>
       </c>
       <c r="B329" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C329" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="330" spans="1:3" x14ac:dyDescent="0.25">
@@ -6193,10 +6193,10 @@
         <v>46532</v>
       </c>
       <c r="B330" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C330" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.25">
@@ -6204,10 +6204,10 @@
         <v>46533</v>
       </c>
       <c r="B331" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C331" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.25">
@@ -6215,10 +6215,10 @@
         <v>46534</v>
       </c>
       <c r="B332" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C332" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.25">
@@ -6248,10 +6248,10 @@
         <v>46537</v>
       </c>
       <c r="B335" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C335" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.25">
@@ -6259,10 +6259,10 @@
         <v>46538</v>
       </c>
       <c r="B336" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C336" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.25">
@@ -6281,10 +6281,10 @@
         <v>46540</v>
       </c>
       <c r="B338" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C338" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.25">
@@ -6292,10 +6292,10 @@
         <v>46541</v>
       </c>
       <c r="B339" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C339" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.25">
@@ -6303,10 +6303,10 @@
         <v>46542</v>
       </c>
       <c r="B340" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C340" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.25">
@@ -6314,10 +6314,10 @@
         <v>46543</v>
       </c>
       <c r="B341" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C341" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.25">
@@ -6325,10 +6325,10 @@
         <v>46544</v>
       </c>
       <c r="B342" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C342" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.25">
@@ -6336,10 +6336,10 @@
         <v>46545</v>
       </c>
       <c r="B343" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C343" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.25">
@@ -6347,10 +6347,10 @@
         <v>46546</v>
       </c>
       <c r="B344" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C344" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.25">
@@ -6380,10 +6380,10 @@
         <v>46549</v>
       </c>
       <c r="B347" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C347" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="348" spans="1:3" x14ac:dyDescent="0.25">
@@ -6391,10 +6391,10 @@
         <v>46550</v>
       </c>
       <c r="B348" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C348" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="349" spans="1:3" x14ac:dyDescent="0.25">
@@ -6413,10 +6413,10 @@
         <v>46552</v>
       </c>
       <c r="B350" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C350" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="351" spans="1:3" x14ac:dyDescent="0.25">
@@ -6424,10 +6424,10 @@
         <v>46553</v>
       </c>
       <c r="B351" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C351" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="352" spans="1:3" x14ac:dyDescent="0.25">
@@ -6435,10 +6435,10 @@
         <v>46554</v>
       </c>
       <c r="B352" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C352" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.25">
@@ -6446,10 +6446,10 @@
         <v>46555</v>
       </c>
       <c r="B353" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C353" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="354" spans="1:3" x14ac:dyDescent="0.25">
@@ -6457,10 +6457,10 @@
         <v>46556</v>
       </c>
       <c r="B354" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C354" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="355" spans="1:3" x14ac:dyDescent="0.25">
@@ -6468,10 +6468,10 @@
         <v>46557</v>
       </c>
       <c r="B355" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C355" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="356" spans="1:3" x14ac:dyDescent="0.25">
@@ -6512,10 +6512,10 @@
         <v>46561</v>
       </c>
       <c r="B359" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C359" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="360" spans="1:3" x14ac:dyDescent="0.25">
@@ -6523,10 +6523,10 @@
         <v>46562</v>
       </c>
       <c r="B360" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C360" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="361" spans="1:3" x14ac:dyDescent="0.25">
@@ -6545,10 +6545,10 @@
         <v>46564</v>
       </c>
       <c r="B362" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C362" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.25">
@@ -6556,10 +6556,10 @@
         <v>46565</v>
       </c>
       <c r="B363" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C363" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.25">
@@ -6567,10 +6567,10 @@
         <v>46566</v>
       </c>
       <c r="B364" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C364" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.25">
@@ -6578,10 +6578,10 @@
         <v>46567</v>
       </c>
       <c r="B365" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C365" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.25">
@@ -6589,10 +6589,10 @@
         <v>46568</v>
       </c>
       <c r="B366" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C366" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Support split months (e.g. Body/IR = first half Body, second half IR)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017xi9tmff2aXUsJqNMSBAwk
</commit_message>
<xml_diff>
--- a/templates/SGUMC_Radiology_Schedule_Sample.xlsx
+++ b/templates/SGUMC_Radiology_Schedule_Sample.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="89">
   <si>
     <t>ResidentID</t>
   </si>
@@ -238,10 +238,16 @@
     <t>Post-Call</t>
   </si>
   <si>
+    <t>IR/Body</t>
+  </si>
+  <si>
     <t>Elective</t>
   </si>
   <si>
     <t>Vascular</t>
+  </si>
+  <si>
+    <t>Body/IR</t>
   </si>
   <si>
     <t>Start Date</t>
@@ -1666,7 +1672,7 @@
         <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="G4" t="s">
         <v>70</v>
@@ -1690,7 +1696,7 @@
         <v>73</v>
       </c>
       <c r="N4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1731,7 +1737,7 @@
         <v>73</v>
       </c>
       <c r="M5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N5" t="s">
         <v>64</v>
@@ -1772,7 +1778,7 @@
         <v>73</v>
       </c>
       <c r="L6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M6" t="s">
         <v>64</v>
@@ -1798,7 +1804,7 @@
         <v>71</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="G7" t="s">
         <v>65</v>
@@ -1813,7 +1819,7 @@
         <v>73</v>
       </c>
       <c r="K7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L7" t="s">
         <v>64</v>
@@ -1854,7 +1860,7 @@
         <v>73</v>
       </c>
       <c r="J8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K8" t="s">
         <v>64</v>
@@ -2255,13 +2261,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -2278,7 +2284,7 @@
         <v>46217</v>
       </c>
       <c r="E2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -2295,7 +2301,7 @@
         <v>46377</v>
       </c>
       <c r="E3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2312,7 +2318,7 @@
         <v>46248</v>
       </c>
       <c r="E4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -2329,7 +2335,7 @@
         <v>46316</v>
       </c>
       <c r="E5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2346,7 +2352,7 @@
         <v>46521</v>
       </c>
       <c r="E6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2363,7 +2369,7 @@
         <v>46286</v>
       </c>
       <c r="E7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2380,7 +2386,7 @@
         <v>46460</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2397,7 +2403,7 @@
         <v>46559</v>
       </c>
       <c r="E9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2414,7 +2420,7 @@
         <v>46401</v>
       </c>
       <c r="E10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2431,7 +2437,7 @@
         <v>46498</v>
       </c>
       <c r="E11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2448,7 +2454,7 @@
         <v>46340</v>
       </c>
       <c r="E12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -2465,7 +2471,7 @@
         <v>46439</v>
       </c>
       <c r="E13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -2482,7 +2488,7 @@
         <v>46217</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -2499,7 +2505,7 @@
         <v>46377</v>
       </c>
       <c r="E15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -2516,7 +2522,7 @@
         <v>46309</v>
       </c>
       <c r="E16" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -2533,7 +2539,7 @@
         <v>46310</v>
       </c>
       <c r="E17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -2550,7 +2556,7 @@
         <v>46286</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2571,13 +2577,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>